<commit_message>
feat(admin): search box on the Registered Languages card
Option A of the Registered Languages search decision (v1, 2026-10-30):
a browser-only filter over the already-loaded language list, no API call.

- Matches English name, code and native label; any part, case-insensitive.
- "N active" keeps counting every language, not just the shown rows.
- "No languages match …" line when nothing matches; ✕ clears the search.
- Toggling a language while filtered keeps the search text.
- Same look as the Feed Selection "Find Feeds" bar.
- 3 new labels in ui-labels.xlsx (machine-translated; need native review).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/src/lib/data/ui-labels.xlsx
+++ b/frontend/src/lib/data/ui-labels.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12698" uniqueCount="11029">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12740" uniqueCount="11068">
   <si>
     <t>English</t>
   </si>
@@ -33226,6 +33226,123 @@
   </si>
   <si>
     <t>Herreegni kun yeroof cufameera. Booda irra deebi'ii yaali ykn PIN jijjiiri.</t>
+  </si>
+  <si>
+    <t>Search languages</t>
+  </si>
+  <si>
+    <t>भाषाएँ खोजें</t>
+  </si>
+  <si>
+    <t>Maghanap ng wika</t>
+  </si>
+  <si>
+    <t>Cari bahasa</t>
+  </si>
+  <si>
+    <t>ค้นหาภาษา</t>
+  </si>
+  <si>
+    <t>Tìm ngôn ngữ</t>
+  </si>
+  <si>
+    <t>ভাষা খুঁজুন</t>
+  </si>
+  <si>
+    <t>भाषा खोज्नुहोस्</t>
+  </si>
+  <si>
+    <t>ቋንቋዎችን ይፈልጉ</t>
+  </si>
+  <si>
+    <t>Afaanota barbaadi</t>
+  </si>
+  <si>
+    <t>ቋንቋታት ድለ</t>
+  </si>
+  <si>
+    <t>Rechercher des langues</t>
+  </si>
+  <si>
+    <t>البحث عن اللغات</t>
+  </si>
+  <si>
+    <t>Search by name or code — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>नाम या कोड से खोजें — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>Maghanap ayon sa pangalan o code — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>Cari berdasarkan nama atau kode — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>ค้นหาตามชื่อหรือรหัส — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>Tìm theo tên hoặc mã — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>নাম বা কোড দিয়ে খুঁজুন — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>नाम वा कोडबाट खोज्नुहोस् — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>በስም ወይም በኮድ ይፈልጉ — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>Maqaa ykn koodiidhaan barbaadi — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>ብሽም ወይ ብኮድ ድለ — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>Rechercher par nom ou code — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>ابحث بالاسم أو الرمز — Hindi, hi…</t>
+  </si>
+  <si>
+    <t>No languages match “${query}”</t>
+  </si>
+  <si>
+    <t>“${query}” से कोई भाषा मेल नहीं खाती</t>
+  </si>
+  <si>
+    <t>Walang wikang tumutugma sa “${query}”</t>
+  </si>
+  <si>
+    <t>Tidak ada bahasa yang cocok dengan “${query}”</t>
+  </si>
+  <si>
+    <t>ไม่มีภาษาที่ตรงกับ “${query}”</t>
+  </si>
+  <si>
+    <t>Không có ngôn ngữ nào khớp với “${query}”</t>
+  </si>
+  <si>
+    <t>“${query}”-এর সাথে কোনো ভাষা মেলেনি</t>
+  </si>
+  <si>
+    <t>“${query}” सँग कुनै भाषा मेल खाएन</t>
+  </si>
+  <si>
+    <t>ከ“${query}” ጋር የሚዛመድ ቋንቋ የለም</t>
+  </si>
+  <si>
+    <t>Afaan “${query}” waliin walsimu hin jiru</t>
+  </si>
+  <si>
+    <t>ምስ “${query}” ዝሰማማዕ ቋንቋ የለን</t>
+  </si>
+  <si>
+    <t>Aucune langue ne correspond à « ${query} »</t>
+  </si>
+  <si>
+    <t>لا توجد لغة تطابق “${query}”</t>
   </si>
 </sst>
 </file>
@@ -33612,7 +33729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N907"/>
+  <dimension ref="A1:N910"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="48" style="1" customWidth="1"/>
@@ -73527,8 +73644,140 @@
         <v>10748</v>
       </c>
     </row>
+    <row r="908" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A908" s="1" t="s">
+        <v>11029</v>
+      </c>
+      <c r="B908" s="1" t="s">
+        <v>11030</v>
+      </c>
+      <c r="C908" s="1" t="s">
+        <v>11031</v>
+      </c>
+      <c r="D908" s="1" t="s">
+        <v>11032</v>
+      </c>
+      <c r="E908" s="1" t="s">
+        <v>11033</v>
+      </c>
+      <c r="F908" s="1" t="s">
+        <v>11034</v>
+      </c>
+      <c r="G908" s="1" t="s">
+        <v>11035</v>
+      </c>
+      <c r="H908" s="1" t="s">
+        <v>11036</v>
+      </c>
+      <c r="I908" s="1" t="s">
+        <v>11037</v>
+      </c>
+      <c r="J908" s="1" t="s">
+        <v>11038</v>
+      </c>
+      <c r="K908" s="1" t="s">
+        <v>11039</v>
+      </c>
+      <c r="L908" s="1" t="s">
+        <v>11040</v>
+      </c>
+      <c r="M908" s="1" t="s">
+        <v>11041</v>
+      </c>
+      <c r="N908" s="1" t="s">
+        <v>7194</v>
+      </c>
+    </row>
+    <row r="909" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A909" s="1" t="s">
+        <v>11042</v>
+      </c>
+      <c r="B909" s="1" t="s">
+        <v>11043</v>
+      </c>
+      <c r="C909" s="1" t="s">
+        <v>11044</v>
+      </c>
+      <c r="D909" s="1" t="s">
+        <v>11045</v>
+      </c>
+      <c r="E909" s="1" t="s">
+        <v>11046</v>
+      </c>
+      <c r="F909" s="1" t="s">
+        <v>11047</v>
+      </c>
+      <c r="G909" s="1" t="s">
+        <v>11048</v>
+      </c>
+      <c r="H909" s="1" t="s">
+        <v>11049</v>
+      </c>
+      <c r="I909" s="1" t="s">
+        <v>11050</v>
+      </c>
+      <c r="J909" s="1" t="s">
+        <v>11051</v>
+      </c>
+      <c r="K909" s="1" t="s">
+        <v>11052</v>
+      </c>
+      <c r="L909" s="1" t="s">
+        <v>11053</v>
+      </c>
+      <c r="M909" s="1" t="s">
+        <v>11054</v>
+      </c>
+      <c r="N909" s="1" t="s">
+        <v>7194</v>
+      </c>
+    </row>
+    <row r="910" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A910" s="1" t="s">
+        <v>11055</v>
+      </c>
+      <c r="B910" s="1" t="s">
+        <v>11056</v>
+      </c>
+      <c r="C910" s="1" t="s">
+        <v>11057</v>
+      </c>
+      <c r="D910" s="1" t="s">
+        <v>11058</v>
+      </c>
+      <c r="E910" s="1" t="s">
+        <v>11059</v>
+      </c>
+      <c r="F910" s="1" t="s">
+        <v>11060</v>
+      </c>
+      <c r="G910" s="1" t="s">
+        <v>11061</v>
+      </c>
+      <c r="H910" s="1" t="s">
+        <v>11062</v>
+      </c>
+      <c r="I910" s="1" t="s">
+        <v>11063</v>
+      </c>
+      <c r="J910" s="1" t="s">
+        <v>11064</v>
+      </c>
+      <c r="K910" s="1" t="s">
+        <v>11065</v>
+      </c>
+      <c r="L910" s="1" t="s">
+        <v>11066</v>
+      </c>
+      <c r="M910" s="1" t="s">
+        <v>11067</v>
+      </c>
+      <c r="N910" s="1" t="s">
+        <v>7194</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>